<commit_message>
"First tier" transformers optimized.
</commit_message>
<xml_diff>
--- a/logs/log_durations/log_durations.xlsx
+++ b/logs/log_durations/log_durations.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="68">
+  <fonts count="75">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -292,6 +292,34 @@
     <font>
       <b val="1"/>
       <color rgb="00853A3A"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00826565"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="003A3A3A"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00807777"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00222222"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F0F0F"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002A2A2A"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00826464"/>
     </font>
   </fonts>
   <fills count="2">
@@ -440,7 +468,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,18 +535,25 @@
     <xf numFmtId="10" fontId="53" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="60" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="61" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="56" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="62" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="68" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="54" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="69" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="55" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="63" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="56" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="70" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="71" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="64" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="72" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="57" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="65" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="73" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="58" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="66" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="59" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="67" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="74" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -893,7 +928,7 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
   </cols>
@@ -2020,6 +2055,16 @@
           <t>09-maps Change %</t>
         </is>
       </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>10-transformers 1</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>10-transformers 1 Change %</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2039,6 +2084,12 @@
       <c r="E42" s="64" t="n">
         <v>0.1428571428571428</v>
       </c>
+      <c r="F42" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="G42" s="23" t="n">
+        <v>-0.5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2058,6 +2109,12 @@
       <c r="E43" s="65" t="n">
         <v>0.008620689655172414</v>
       </c>
+      <c r="F43" s="5" t="n">
+        <v>541</v>
+      </c>
+      <c r="G43" s="66" t="n">
+        <v>-0.1760869565217391</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2077,6 +2134,12 @@
       <c r="E44" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2096,6 +2159,12 @@
       <c r="E45" s="23" t="n">
         <v>-0.5185185185185185</v>
       </c>
+      <c r="F45" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="G45" s="21" t="n">
+        <v>0.3658536585365854</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2112,8 +2181,14 @@
       <c r="D46" s="5" t="n">
         <v>577</v>
       </c>
-      <c r="E46" s="66" t="n">
+      <c r="E46" s="67" t="n">
         <v>-0.2462203023758099</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>534</v>
+      </c>
+      <c r="G46" s="68" t="n">
+        <v>0.07452339688041594</v>
       </c>
     </row>
     <row r="47">
@@ -2134,6 +2209,12 @@
       <c r="E47" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2153,6 +2234,12 @@
       <c r="E48" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2163,7 +2250,7 @@
       <c r="B49" s="5" t="n">
         <v>216</v>
       </c>
-      <c r="C49" s="67" t="n">
+      <c r="C49" s="69" t="n">
         <v>0.009174311926605505</v>
       </c>
       <c r="D49" s="5" t="n">
@@ -2172,6 +2259,12 @@
       <c r="E49" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F49" s="5" t="n">
+        <v>275</v>
+      </c>
+      <c r="G49" s="70" t="n">
+        <v>-0.2731481481481481</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2191,6 +2284,12 @@
       <c r="E50" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2210,6 +2309,12 @@
       <c r="E51" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2220,7 +2325,7 @@
       <c r="B52" s="5" t="n">
         <v>327</v>
       </c>
-      <c r="C52" s="68" t="n">
+      <c r="C52" s="71" t="n">
         <v>-0.06862745098039216</v>
       </c>
       <c r="D52" s="5" t="n">
@@ -2229,6 +2334,12 @@
       <c r="E52" s="42" t="n">
         <v>-0.1498470948012232</v>
       </c>
+      <c r="F52" s="5" t="n">
+        <v>347</v>
+      </c>
+      <c r="G52" s="68" t="n">
+        <v>0.07712765957446809</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2245,8 +2356,14 @@
       <c r="D53" s="5" t="n">
         <v>782</v>
       </c>
-      <c r="E53" s="69" t="n">
+      <c r="E53" s="72" t="n">
         <v>-0.225705329153605</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>763</v>
+      </c>
+      <c r="G53" s="73" t="n">
+        <v>0.02429667519181586</v>
       </c>
     </row>
     <row r="54">
@@ -2258,7 +2375,7 @@
       <c r="B54" s="5" t="n">
         <v>82</v>
       </c>
-      <c r="C54" s="70" t="n">
+      <c r="C54" s="66" t="n">
         <v>-0.09333333333333334</v>
       </c>
       <c r="D54" s="5" t="n">
@@ -2267,6 +2384,12 @@
       <c r="E54" s="21" t="n">
         <v>0.1951219512195122</v>
       </c>
+      <c r="F54" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="G54" s="74" t="n">
+        <v>-0.3636363636363636</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2283,8 +2406,14 @@
       <c r="D55" s="5" t="n">
         <v>4992</v>
       </c>
-      <c r="E55" s="71" t="n">
+      <c r="E55" s="75" t="n">
         <v>0.07743485492515247</v>
+      </c>
+      <c r="F55" s="5" t="n">
+        <v>7195</v>
+      </c>
+      <c r="G55" s="76" t="n">
+        <v>-0.4413060897435898</v>
       </c>
     </row>
     <row r="56">
@@ -2296,14 +2425,20 @@
       <c r="B56" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="C56" s="72" t="n">
+      <c r="C56" s="77" t="n">
         <v>0.02777777777777778</v>
       </c>
       <c r="D56" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="E56" s="73" t="n">
+      <c r="E56" s="78" t="n">
         <v>-0.02857142857142857</v>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="G56" s="79" t="n">
+        <v>-0.3333333333333333</v>
       </c>
     </row>
     <row r="57">
@@ -2315,14 +2450,20 @@
       <c r="B57" s="5" t="n">
         <v>929</v>
       </c>
-      <c r="C57" s="74" t="n">
+      <c r="C57" s="80" t="n">
         <v>0.01484623541887593</v>
       </c>
       <c r="D57" s="5" t="n">
         <v>830</v>
       </c>
-      <c r="E57" s="75" t="n">
+      <c r="E57" s="81" t="n">
         <v>0.1065662002152852</v>
+      </c>
+      <c r="F57" s="5" t="n">
+        <v>825</v>
+      </c>
+      <c r="G57" s="48" t="n">
+        <v>0.006024096385542169</v>
       </c>
     </row>
     <row r="58">
@@ -2334,14 +2475,20 @@
       <c r="B58" s="29" t="n">
         <v>340</v>
       </c>
-      <c r="C58" s="76" t="n">
+      <c r="C58" s="82" t="n">
         <v>-0.1184210526315789</v>
       </c>
       <c r="D58" s="29" t="n">
         <v>304</v>
       </c>
-      <c r="E58" s="77" t="n">
+      <c r="E58" s="83" t="n">
         <v>0.1058823529411765</v>
+      </c>
+      <c r="F58" s="29" t="n">
+        <v>280</v>
+      </c>
+      <c r="G58" s="84" t="n">
+        <v>0.07894736842105263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>